<commit_message>
Finance & Users module pending in vendors
</commit_message>
<xml_diff>
--- a/media/parts/part_import_template.xlsx
+++ b/media/parts/part_import_template.xlsx
@@ -453,7 +453,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S2"/>
+  <dimension ref="A1:R2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -565,11 +565,6 @@
       </c>
       <c r="R1" s="4" t="inlineStr">
         <is>
-          <t>Compatible Vehicles</t>
-        </is>
-      </c>
-      <c r="S1" s="4" t="inlineStr">
-        <is>
           <t>Image URL</t>
         </is>
       </c>
@@ -649,11 +644,6 @@
         </is>
       </c>
       <c r="R2" t="inlineStr">
-        <is>
-          <t>Toyota Hilux, Toyota Fortuner</t>
-        </is>
-      </c>
-      <c r="S2" t="inlineStr">
         <is>
           <t>https://example.com/images/brake-pad.jpg</t>
         </is>

</xml_diff>